<commit_message>
Actualizaciones automáticas (versión 0.2.0)
- Plugins updater y process: al abrir, la app busca una versión nueva,
  pregunta, muestra el progreso, instala y se reinicia.
- Prueba se actualiza desde la release "canal-test"; producción desde la
  última Release. CI publica instaladores firmados en cada canal.
- Versión única en package.json (0.2.0), visible al pie del menú.
- Solo instalador NSIS. La plantilla de alumnos usa un teléfono ficticio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_alumnos.xlsx
+++ b/plantillas/plantilla_alumnos.xlsx
@@ -44,7 +44,7 @@
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Característica + número, sin 0 ni 15. Ej: 3400445198</t>
+          <t>Característica + número, sin 0 ni 15. Ej: 3400123456</t>
         </r>
       </text>
     </comment>
@@ -138,7 +138,7 @@
     <t>Obligatorios. En columnas separadas (no «Apellido, Nombre» en una sola).</t>
   </si>
   <si>
-    <t>Característica + número, SIN 0 y SIN 15. Ej: 3400445198 (no 03400 15 445198). Es el número al que llegan los recibos.</t>
+    <t>Característica + número, SIN 0 y SIN 15. Ej: 3400123456 (no 03400 15 445198). Es el número al que llegan los recibos.</t>
   </si>
   <si>
     <t>Curso / Otro curso</t>
@@ -171,7 +171,7 @@
     <t>28456123</t>
   </si>
   <si>
-    <t>3400445198</t>
+    <t>3400123456</t>
   </si>
   <si>
     <t>Segundo</t>
@@ -6199,11 +6199,11 @@
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <dataValidations count="8">
-    <dataValidation type="textLength" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Revisá el teléfono" error="Debe tener 10 dígitos: característica + número, sin 0 ni 15 (ej: 3400445198)." sqref="D10:D501">
+    <dataValidation type="textLength" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Revisá el teléfono" error="Debe tener 10 dígitos: característica + número, sin 0 ni 15 (ej: 3400123456)." sqref="D10:D501">
       <formula1>10</formula1>
       <formula2>13</formula2>
     </dataValidation>
-    <dataValidation type="textLength" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Revisá el teléfono" error="Debe tener 10 dígitos: característica + número, sin 0 ni 15 (ej: 3400445198)." sqref="D2:D501">
+    <dataValidation type="textLength" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Revisá el teléfono" error="Debe tener 10 dígitos: característica + número, sin 0 ni 15 (ej: 3400123456)." sqref="D2:D501">
       <formula1>10</formula1>
       <formula2>13</formula2>
     </dataValidation>

</xml_diff>